<commit_message>
Aggiornamento database SAFIT del 25/02/2026 ore 10:39:57,35
</commit_message>
<xml_diff>
--- a/utenti.xlsx
+++ b/utenti.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\git-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5101E39-FEEC-46A7-A4A6-E9F39AE906A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1740674D-CF5A-4227-8B0A-78DB43E1AB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>username</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>C000744 - SPIRALE SRL</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
 </sst>
 </file>
@@ -519,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E837CC2E-FFAA-493E-9E03-C350178C8C16}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19.28515625" customWidth="1"/>
@@ -611,6 +614,17 @@
         <v>46078</v>
       </c>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Aggiornamento dati 26/02/2026 12:01:13,62
</commit_message>
<xml_diff>
--- a/utenti.xlsx
+++ b/utenti.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\git-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1740674D-CF5A-4227-8B0A-78DB43E1AB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC719A6-80ED-41EB-93C8-CCD42494C9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
+    <workbookView xWindow="1380" yWindow="3600" windowWidth="15030" windowHeight="12000" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>username</t>
   </si>
@@ -95,7 +95,10 @@
     <t>C000744 - SPIRALE SRL</t>
   </si>
   <si>
-    <t>test</t>
+    <t>nikola</t>
+  </si>
+  <si>
+    <t>nik001</t>
   </si>
 </sst>
 </file>
@@ -169,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -186,6 +189,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -619,10 +625,13 @@
         <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
+      </c>
+      <c r="D7" s="8">
+        <v>46078</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aggiornamento dati 26/02/2026 14:30:43,95
</commit_message>
<xml_diff>
--- a/utenti.xlsx
+++ b/utenti.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\git-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4EEC14-7352-4D24-B35D-5F6ECFFE5275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F310C3F-8A87-4DB6-9159-30F45335E322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="3600" windowWidth="15030" windowHeight="12000" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
+    <workbookView xWindow="5880" yWindow="1995" windowWidth="15030" windowHeight="12000" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>username</t>
   </si>
@@ -95,17 +95,23 @@
     <t>C000744 - SPIRALE SRL</t>
   </si>
   <si>
-    <t>nikola</t>
-  </si>
-  <si>
-    <t>nik001</t>
+    <t>Nikola</t>
+  </si>
+  <si>
+    <t>Nik001</t>
+  </si>
+  <si>
+    <t>valentina</t>
+  </si>
+  <si>
+    <t>val222</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,6 +120,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -172,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -187,11 +200,10 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -528,7 +540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E837CC2E-FFAA-493E-9E03-C350178C8C16}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19.28515625" customWidth="1"/>
@@ -537,16 +549,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>15</v>
       </c>
     </row>
@@ -575,7 +587,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="5">
-        <v>46077</v>
+        <v>46078</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -589,10 +601,10 @@
         <v>11</v>
       </c>
       <c r="D4" s="5">
-        <v>46077</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>46079</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
@@ -602,39 +614,54 @@
       <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="6">
-        <v>46078</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="D5" s="5">
+        <v>46080</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="6">
-        <v>46078</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="D6" s="5">
+        <v>46081</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="8">
-        <v>46078</v>
+      <c r="D7" s="5">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="5">
+        <v>46083</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Aggiornamento dati 26/02/2026 14:49:15,01
</commit_message>
<xml_diff>
--- a/utenti.xlsx
+++ b/utenti.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\git-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F310C3F-8A87-4DB6-9159-30F45335E322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E9F9D7-4FC6-4B2C-83BA-8B22153BDA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5880" yWindow="1995" windowWidth="15030" windowHeight="12000" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
+    <workbookView xWindow="14775" yWindow="3405" windowWidth="9240" windowHeight="8730" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -98,13 +98,13 @@
     <t>Nikola</t>
   </si>
   <si>
-    <t>Nik001</t>
-  </si>
-  <si>
     <t>valentina</t>
   </si>
   <si>
     <t>val222</t>
+  </si>
+  <si>
+    <t>Nik789</t>
   </si>
 </sst>
 </file>
@@ -633,11 +633,11 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>20</v>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -648,10 +648,10 @@
     </row>
     <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Aggiornamento dati 26/02/2026 15:15:16,74
</commit_message>
<xml_diff>
--- a/utenti.xlsx
+++ b/utenti.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\git-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E9F9D7-4FC6-4B2C-83BA-8B22153BDA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3FE09FA-B128-4569-B10E-69F032DC636D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14775" yWindow="3405" windowWidth="9240" windowHeight="8730" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>username</t>
   </si>
@@ -105,6 +105,12 @@
   </si>
   <si>
     <t>Nik789</t>
+  </si>
+  <si>
+    <t>pippo</t>
+  </si>
+  <si>
+    <t>pip963</t>
   </si>
 </sst>
 </file>
@@ -540,7 +546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E837CC2E-FFAA-493E-9E03-C350178C8C16}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19.28515625" customWidth="1"/>
@@ -660,6 +666,20 @@
         <v>46083</v>
       </c>
     </row>
+    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="5">
+        <v>46084</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Aggiornamento dati locale 27/02/2026  8:55:05,04
</commit_message>
<xml_diff>
--- a/utenti.xlsx
+++ b/utenti.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\git-files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Venezian.Denis\Desktop\python_access_sql\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3FE09FA-B128-4569-B10E-69F032DC636D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B7DA4F-DCBE-4E9A-B31F-AF81692D102D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{38FE3314-E022-4CA1-9956-19B554EBCB7E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>username</t>
   </si>
@@ -56,15 +56,6 @@
     <t>TUTTI</t>
   </si>
   <si>
-    <t>gar_demo</t>
-  </si>
-  <si>
-    <t>gar789</t>
-  </si>
-  <si>
-    <t>C000161 - GARSPORT SRL</t>
-  </si>
-  <si>
     <t>annic_demo</t>
   </si>
   <si>
@@ -95,29 +86,23 @@
     <t>C000744 - SPIRALE SRL</t>
   </si>
   <si>
-    <t>Nikola</t>
+    <t>nikola</t>
+  </si>
+  <si>
+    <t>nikola2026</t>
   </si>
   <si>
     <t>valentina</t>
   </si>
   <si>
-    <t>val222</t>
-  </si>
-  <si>
-    <t>Nik789</t>
-  </si>
-  <si>
-    <t>pippo</t>
-  </si>
-  <si>
-    <t>pip963</t>
+    <t>vale2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,13 +111,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -191,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -206,10 +184,11 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -546,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E837CC2E-FFAA-493E-9E03-C350178C8C16}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="19.28515625" customWidth="1"/>
@@ -555,17 +534,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
-        <v>15</v>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -584,104 +563,75 @@
     </row>
     <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3" s="5">
-        <v>46078</v>
+        <v>46077</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="5">
+        <v>46077</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5">
-        <v>46079</v>
+      <c r="D5" s="6">
+        <v>46078</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="5">
-        <v>46080</v>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6">
+        <v>46078</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="5">
-        <v>46081</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="B7" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="5">
-        <v>46082</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="5">
-        <v>46083</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="5">
-        <v>46084</v>
+      <c r="D7" s="8">
+        <v>46078</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>